<commit_message>
Added new error message
</commit_message>
<xml_diff>
--- a/jeaf-generator-messages/src/main/resources/JEAFGeneratorMessages.xlsx
+++ b/jeaf-generator-messages/src/main/resources/JEAFGeneratorMessages.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tillmann.schall/Projects/JEAF/jeaf-generator-messages/jeaf-generator-messages/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5270039F-D62B-A04C-B74F-4AB91CF1DBC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFCF081-8A51-8044-B76C-7D6F7BAE686F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25620" yWindow="640" windowWidth="51160" windowHeight="28140" activeTab="2" xr2:uid="{ADB42BFB-6EC0-410A-8CB1-9C298A092AA4}"/>
   </bookViews>
@@ -281,7 +281,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="336">
   <si>
     <t>Class-Info</t>
   </si>
@@ -1290,6 +1290,16 @@
   </si>
   <si>
     <t>When working with bean parameters, it is generally expected that every property of a bean parameter class represents a header, path, query, or cookie parameter. In cases where a bean parameter class also includes simple properties for other purposes, those properties must be explicitly marked as “not a REST parameter” using stereotype «NoRESTParam».</t>
+  </si>
+  <si>
+    <t>TOO_MANY_COMPATIBILITY_INFOS</t>
+  </si>
+  <si>
+    <t>So called compatibility groups can be used to simplify handling of deprecation and breaking changes message. One part of this is defining compatibility info for a compatibility group.
+However you can not define more the one compatibility info for a compatibility group</t>
+  </si>
+  <si>
+    <t>«CompatibilityGroup» ''{0}'' has multiple «CompatibilityInfo» definitions associated ({1}). Please make sure that there is not more than one.</t>
   </si>
 </sst>
 </file>
@@ -4579,9 +4589,24 @@
         <v>331</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7" ht="80" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>9187</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
@@ -4645,7 +4670,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A101" xr:uid="{AACEF8C0-EC92-4686-A8C3-E4036D94D483}">
       <formula1>0</formula1>
     </dataValidation>
@@ -4658,7 +4683,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EA474BAA-D9F0-48C4-BFC6-D7532DADFCD0}">
           <x14:formula1>
             <xm:f>'Predefined-Values'!$C$4:$C$5</xm:f>

</xml_diff>